<commit_message>
changes for mdms migration
</commit_message>
<xml_diff>
--- a/jupyter/dataloader/templates/Employee_Master_Dynamic_statea.xlsx
+++ b/jupyter/dataloader/templates/Employee_Master_Dynamic_statea.xlsx
@@ -957,15 +957,19 @@
       <c r="N2" s="3" t="n">
         <v>45463</v>
       </c>
-      <c r="O2" s="12" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
+      <c r="O2" s="11" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>202</v>
-      </c>
-      <c r="Q2" t="inlineStr"/>
+        <v>400</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>An error occurred while accessing a underlying resource</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="M3" s="3" t="n"/>

</xml_diff>